<commit_message>
Add a 12 hour row to the storms-only example
Every included row was 24 hours, which sits above the example project's 9-18
hour GSDM/GTSMR changeover band, so apply_extreme_method returned GTSMR by
rule and the random branch never ran. The 6 hour row (excluded by default) is
below the band and equally deterministic. Nothing in the example therefore
exercised the per-realisation sampling of the extreme method, or the separate
sampling of the spatial method that goes with it.

A 12 hour row lands mid-band. On its mcdf the ARR realisations split evenly
between GSDM and GTSMR spatial methods while those that sampled an extreme
method keep it -- the behaviour 9ea16a2 introduced, which no example covered.

The row goes in make_example_configs.py, which generates both workbooks;
SimsList_routing.xlsx is re-serialised but its content is unchanged.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KVm3831QHViNNaoWidTD2y
</commit_message>
<xml_diff>
--- a/example_project/SimsList_storms.xlsx
+++ b/example_project/SimsList_storms.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -799,7 +799,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -808,7 +808,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -822,7 +822,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -873,15 +873,106 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
+          <t>results/storms_12h_gwl0_log.txt</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>results/storms_12h_gwl0</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Inside the 9-18 h GSDM/GTSMR changeover band, so both the storm method and the spatial method are sampled per realisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>monte carlo</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>storms only</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>fsv</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>sim_options/lake_conditions/lake_config.json</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>sim_options/focal_locations/SYNTHETIC_dam_subcatchments.csv</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>sim_options/mc_config.json</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>30</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>pb</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
           <t>results/storms_6h_gwl0_log.txt</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>results/storms_6h_gwl0</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>A short duration, so GSDM patterns are sampled. Set Include to yes to run</t>
         </is>

</xml_diff>